<commit_message>
Update drivebonus template as requested by user
</commit_message>
<xml_diff>
--- a/public/templates/drivebonus_template.xlsx
+++ b/public/templates/drivebonus_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\wordtoexcel\staff_manager\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56BCF40F-C7CB-49DD-9A4E-E9774BE0742C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{121A8E1C-6EC0-466B-81B6-BA4564DEB0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{FE9DB102-5480-4C6F-9AE4-967FBD7E5687}"/>
+    <workbookView xWindow="1245" yWindow="750" windowWidth="27150" windowHeight="18705" activeTab="1" xr2:uid="{FE9DB102-5480-4C6F-9AE4-967FBD7E5687}"/>
   </bookViews>
   <sheets>
     <sheet name="正駕" sheetId="1" r:id="rId1"/>
@@ -282,9 +282,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>承辦人</t>
-  </si>
-  <si>
     <t>區隊長</t>
   </si>
   <si>
@@ -322,6 +319,10 @@
   </si>
   <si>
     <t>____{{year}}____年_{{month}}_月份</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>領班長</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -851,6 +852,33 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -911,40 +939,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1274,153 +1275,153 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="44.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
-      <c r="S1" s="26"/>
-      <c r="T1" s="26"/>
-      <c r="U1" s="26"/>
-      <c r="V1" s="26"/>
-      <c r="W1" s="26"/>
-      <c r="X1" s="27" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="35"/>
+      <c r="V1" s="35"/>
+      <c r="W1" s="35"/>
+      <c r="X1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="Y1" s="28"/>
-      <c r="Z1" s="28"/>
-      <c r="AA1" s="28"/>
-      <c r="AB1" s="28"/>
-      <c r="AC1" s="28"/>
-      <c r="AD1" s="28"/>
-      <c r="AE1" s="28"/>
-      <c r="AF1" s="28"/>
-      <c r="AG1" s="28"/>
-      <c r="AH1" s="28"/>
-      <c r="AI1" s="28"/>
-      <c r="AJ1" s="28"/>
-      <c r="AK1" s="28"/>
-      <c r="AL1" s="29"/>
+      <c r="Y1" s="37"/>
+      <c r="Z1" s="37"/>
+      <c r="AA1" s="37"/>
+      <c r="AB1" s="37"/>
+      <c r="AC1" s="37"/>
+      <c r="AD1" s="37"/>
+      <c r="AE1" s="37"/>
+      <c r="AF1" s="37"/>
+      <c r="AG1" s="37"/>
+      <c r="AH1" s="37"/>
+      <c r="AI1" s="37"/>
+      <c r="AJ1" s="37"/>
+      <c r="AK1" s="37"/>
+      <c r="AL1" s="38"/>
     </row>
     <row r="2" spans="1:38" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="26"/>
-      <c r="T2" s="26"/>
-      <c r="U2" s="26"/>
-      <c r="V2" s="26"/>
-      <c r="W2" s="26"/>
-      <c r="X2" s="30"/>
-      <c r="Y2" s="31"/>
-      <c r="Z2" s="31"/>
-      <c r="AA2" s="31"/>
-      <c r="AB2" s="31"/>
-      <c r="AC2" s="31"/>
-      <c r="AD2" s="31"/>
-      <c r="AE2" s="31"/>
-      <c r="AF2" s="31"/>
-      <c r="AG2" s="31"/>
-      <c r="AH2" s="31"/>
-      <c r="AI2" s="31"/>
-      <c r="AJ2" s="31"/>
-      <c r="AK2" s="31"/>
-      <c r="AL2" s="32"/>
+      <c r="A2" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
+      <c r="T2" s="35"/>
+      <c r="U2" s="35"/>
+      <c r="V2" s="35"/>
+      <c r="W2" s="35"/>
+      <c r="X2" s="39"/>
+      <c r="Y2" s="40"/>
+      <c r="Z2" s="40"/>
+      <c r="AA2" s="40"/>
+      <c r="AB2" s="40"/>
+      <c r="AC2" s="40"/>
+      <c r="AD2" s="40"/>
+      <c r="AE2" s="40"/>
+      <c r="AF2" s="40"/>
+      <c r="AG2" s="40"/>
+      <c r="AH2" s="40"/>
+      <c r="AI2" s="40"/>
+      <c r="AJ2" s="40"/>
+      <c r="AK2" s="40"/>
+      <c r="AL2" s="41"/>
     </row>
     <row r="3" spans="1:38" s="1" customFormat="1" ht="42.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="40"/>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="40"/>
-      <c r="O3" s="40"/>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="40"/>
-      <c r="R3" s="40"/>
-      <c r="S3" s="40"/>
-      <c r="T3" s="40"/>
-      <c r="U3" s="40"/>
-      <c r="V3" s="40"/>
-      <c r="W3" s="40"/>
-      <c r="X3" s="40"/>
-      <c r="Y3" s="40"/>
-      <c r="Z3" s="40"/>
-      <c r="AA3" s="40"/>
-      <c r="AB3" s="40"/>
-      <c r="AC3" s="40"/>
-      <c r="AD3" s="40"/>
-      <c r="AE3" s="40"/>
-      <c r="AF3" s="40"/>
-      <c r="AG3" s="40"/>
-      <c r="AH3" s="41"/>
-      <c r="AI3" s="42" t="s">
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
+      <c r="L3" s="49"/>
+      <c r="M3" s="49"/>
+      <c r="N3" s="49"/>
+      <c r="O3" s="49"/>
+      <c r="P3" s="49"/>
+      <c r="Q3" s="49"/>
+      <c r="R3" s="49"/>
+      <c r="S3" s="49"/>
+      <c r="T3" s="49"/>
+      <c r="U3" s="49"/>
+      <c r="V3" s="49"/>
+      <c r="W3" s="49"/>
+      <c r="X3" s="49"/>
+      <c r="Y3" s="49"/>
+      <c r="Z3" s="49"/>
+      <c r="AA3" s="49"/>
+      <c r="AB3" s="49"/>
+      <c r="AC3" s="49"/>
+      <c r="AD3" s="49"/>
+      <c r="AE3" s="49"/>
+      <c r="AF3" s="49"/>
+      <c r="AG3" s="49"/>
+      <c r="AH3" s="50"/>
+      <c r="AI3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="AJ3" s="42" t="s">
+      <c r="AJ3" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="AK3" s="42" t="s">
+      <c r="AK3" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="AL3" s="44" t="s">
+      <c r="AL3" s="53" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:38" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="34"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="38"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="47"/>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -1452,20 +1453,20 @@
       <c r="AF4" s="2"/>
       <c r="AG4" s="2"/>
       <c r="AH4" s="2"/>
-      <c r="AI4" s="43"/>
-      <c r="AJ4" s="43"/>
-      <c r="AK4" s="43"/>
-      <c r="AL4" s="45"/>
+      <c r="AI4" s="52"/>
+      <c r="AJ4" s="52"/>
+      <c r="AK4" s="52"/>
+      <c r="AL4" s="54"/>
     </row>
     <row r="5" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="57" t="s">
-        <v>24</v>
+      <c r="A5" s="26" t="s">
+        <v>23</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -1508,7 +1509,7 @@
       <c r="AL5" s="7"/>
     </row>
     <row r="6" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="57"/>
+      <c r="A6" s="26"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="6"/>
@@ -1552,7 +1553,7 @@
       <c r="AL6" s="7"/>
     </row>
     <row r="7" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="57"/>
+      <c r="A7" s="26"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="6"/>
@@ -1596,7 +1597,7 @@
       <c r="AL7" s="7"/>
     </row>
     <row r="8" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="57"/>
+      <c r="A8" s="26"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="6"/>
@@ -1640,7 +1641,7 @@
       <c r="AL8" s="7"/>
     </row>
     <row r="9" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="57"/>
+      <c r="A9" s="26"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="6"/>
@@ -1684,7 +1685,7 @@
       <c r="AL9" s="7"/>
     </row>
     <row r="10" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="57"/>
+      <c r="A10" s="26"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="6"/>
@@ -1728,7 +1729,7 @@
       <c r="AL10" s="7"/>
     </row>
     <row r="11" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="57"/>
+      <c r="A11" s="26"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="6"/>
@@ -1772,7 +1773,7 @@
       <c r="AL11" s="7"/>
     </row>
     <row r="12" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="57"/>
+      <c r="A12" s="26"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="6"/>
@@ -1816,7 +1817,7 @@
       <c r="AL12" s="7"/>
     </row>
     <row r="13" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="57"/>
+      <c r="A13" s="26"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="6"/>
@@ -1860,7 +1861,7 @@
       <c r="AL13" s="7"/>
     </row>
     <row r="14" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="57"/>
+      <c r="A14" s="26"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="6"/>
@@ -1904,86 +1905,86 @@
       <c r="AL14" s="7"/>
     </row>
     <row r="15" spans="1:38" s="8" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="46" t="s">
+      <c r="A15" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="47"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="47"/>
-      <c r="E15" s="47"/>
-      <c r="F15" s="47"/>
-      <c r="G15" s="47"/>
-      <c r="H15" s="47"/>
-      <c r="I15" s="47"/>
-      <c r="J15" s="47"/>
-      <c r="K15" s="47"/>
-      <c r="L15" s="47"/>
-      <c r="M15" s="47"/>
-      <c r="N15" s="47"/>
-      <c r="O15" s="47"/>
-      <c r="P15" s="47"/>
-      <c r="Q15" s="47"/>
-      <c r="R15" s="47"/>
-      <c r="S15" s="47"/>
-      <c r="T15" s="47"/>
-      <c r="U15" s="47"/>
-      <c r="V15" s="47"/>
-      <c r="W15" s="47"/>
-      <c r="X15" s="47"/>
-      <c r="Y15" s="47"/>
-      <c r="Z15" s="47"/>
-      <c r="AA15" s="47"/>
-      <c r="AB15" s="47"/>
-      <c r="AC15" s="47"/>
-      <c r="AD15" s="47"/>
-      <c r="AE15" s="47"/>
-      <c r="AF15" s="47"/>
-      <c r="AG15" s="47"/>
-      <c r="AH15" s="47"/>
-      <c r="AI15" s="47"/>
-      <c r="AJ15" s="47"/>
-      <c r="AK15" s="47"/>
-      <c r="AL15" s="48"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="28"/>
+      <c r="K15" s="28"/>
+      <c r="L15" s="28"/>
+      <c r="M15" s="28"/>
+      <c r="N15" s="28"/>
+      <c r="O15" s="28"/>
+      <c r="P15" s="28"/>
+      <c r="Q15" s="28"/>
+      <c r="R15" s="28"/>
+      <c r="S15" s="28"/>
+      <c r="T15" s="28"/>
+      <c r="U15" s="28"/>
+      <c r="V15" s="28"/>
+      <c r="W15" s="28"/>
+      <c r="X15" s="28"/>
+      <c r="Y15" s="28"/>
+      <c r="Z15" s="28"/>
+      <c r="AA15" s="28"/>
+      <c r="AB15" s="28"/>
+      <c r="AC15" s="28"/>
+      <c r="AD15" s="28"/>
+      <c r="AE15" s="28"/>
+      <c r="AF15" s="28"/>
+      <c r="AG15" s="28"/>
+      <c r="AH15" s="28"/>
+      <c r="AI15" s="28"/>
+      <c r="AJ15" s="28"/>
+      <c r="AK15" s="28"/>
+      <c r="AL15" s="29"/>
     </row>
     <row r="16" spans="1:38" s="8" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A16" s="49"/>
-      <c r="B16" s="50"/>
-      <c r="C16" s="50"/>
-      <c r="D16" s="50"/>
-      <c r="E16" s="50"/>
-      <c r="F16" s="50"/>
-      <c r="G16" s="50"/>
-      <c r="H16" s="50"/>
-      <c r="I16" s="50"/>
-      <c r="J16" s="50"/>
-      <c r="K16" s="50"/>
-      <c r="L16" s="50"/>
-      <c r="M16" s="50"/>
-      <c r="N16" s="50"/>
-      <c r="O16" s="50"/>
-      <c r="P16" s="50"/>
-      <c r="Q16" s="50"/>
-      <c r="R16" s="50"/>
-      <c r="S16" s="50"/>
-      <c r="T16" s="50"/>
-      <c r="U16" s="50"/>
-      <c r="V16" s="50"/>
-      <c r="W16" s="50"/>
-      <c r="X16" s="50"/>
-      <c r="Y16" s="50"/>
-      <c r="Z16" s="50"/>
-      <c r="AA16" s="50"/>
-      <c r="AB16" s="50"/>
-      <c r="AC16" s="50"/>
-      <c r="AD16" s="50"/>
-      <c r="AE16" s="50"/>
-      <c r="AF16" s="50"/>
-      <c r="AG16" s="50"/>
-      <c r="AH16" s="50"/>
-      <c r="AI16" s="50"/>
-      <c r="AJ16" s="50"/>
-      <c r="AK16" s="50"/>
-      <c r="AL16" s="51"/>
+      <c r="A16" s="30"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="31"/>
+      <c r="L16" s="31"/>
+      <c r="M16" s="31"/>
+      <c r="N16" s="31"/>
+      <c r="O16" s="31"/>
+      <c r="P16" s="31"/>
+      <c r="Q16" s="31"/>
+      <c r="R16" s="31"/>
+      <c r="S16" s="31"/>
+      <c r="T16" s="31"/>
+      <c r="U16" s="31"/>
+      <c r="V16" s="31"/>
+      <c r="W16" s="31"/>
+      <c r="X16" s="31"/>
+      <c r="Y16" s="31"/>
+      <c r="Z16" s="31"/>
+      <c r="AA16" s="31"/>
+      <c r="AB16" s="31"/>
+      <c r="AC16" s="31"/>
+      <c r="AD16" s="31"/>
+      <c r="AE16" s="31"/>
+      <c r="AF16" s="31"/>
+      <c r="AG16" s="31"/>
+      <c r="AH16" s="31"/>
+      <c r="AI16" s="31"/>
+      <c r="AJ16" s="31"/>
+      <c r="AK16" s="31"/>
+      <c r="AL16" s="32"/>
     </row>
     <row r="17" spans="1:38" s="12" customFormat="1" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="9" t="s">
@@ -1991,62 +1992,56 @@
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="10" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
-      <c r="H17" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="I17" s="52"/>
-      <c r="J17" s="52"/>
+      <c r="H17" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17" s="33"/>
+      <c r="J17" s="33"/>
       <c r="K17" s="10"/>
       <c r="L17" s="10"/>
       <c r="M17" s="11"/>
       <c r="N17" s="11"/>
       <c r="O17" s="11"/>
-      <c r="P17" s="52" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q17" s="52"/>
-      <c r="R17" s="52"/>
+      <c r="P17" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q17" s="33"/>
+      <c r="R17" s="33"/>
       <c r="S17" s="11"/>
       <c r="T17" s="11"/>
       <c r="U17" s="11"/>
-      <c r="V17" s="52" t="s">
-        <v>17</v>
-      </c>
-      <c r="W17" s="52"/>
-      <c r="X17" s="52"/>
+      <c r="V17" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="W17" s="33"/>
+      <c r="X17" s="33"/>
       <c r="Y17" s="11"/>
       <c r="Z17" s="11"/>
       <c r="AA17" s="11"/>
-      <c r="AB17" s="52" t="s">
-        <v>18</v>
-      </c>
-      <c r="AC17" s="52"/>
-      <c r="AD17" s="52"/>
+      <c r="AB17" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="AC17" s="33"/>
+      <c r="AD17" s="33"/>
       <c r="AE17" s="11"/>
       <c r="AF17" s="11"/>
       <c r="AG17" s="11"/>
-      <c r="AH17" s="52" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI17" s="53"/>
+      <c r="AH17" s="33" t="s">
+        <v>18</v>
+      </c>
+      <c r="AI17" s="34"/>
       <c r="AJ17" s="10"/>
       <c r="AK17" s="10"/>
       <c r="AL17" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A15:AL16"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="P17:R17"/>
-    <mergeCell ref="V17:X17"/>
-    <mergeCell ref="AB17:AD17"/>
-    <mergeCell ref="AH17:AI17"/>
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="X1:AL2"/>
     <mergeCell ref="A2:W2"/>
@@ -2058,6 +2053,12 @@
     <mergeCell ref="AJ3:AJ4"/>
     <mergeCell ref="AK3:AK4"/>
     <mergeCell ref="AL3:AL4"/>
+    <mergeCell ref="A15:AL16"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="P17:R17"/>
+    <mergeCell ref="V17:X17"/>
+    <mergeCell ref="AB17:AD17"/>
+    <mergeCell ref="AH17:AI17"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2086,153 +2087,153 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="44.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
-      <c r="S1" s="26"/>
-      <c r="T1" s="26"/>
-      <c r="U1" s="26"/>
-      <c r="V1" s="26"/>
-      <c r="W1" s="26"/>
-      <c r="X1" s="27" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="35"/>
+      <c r="V1" s="35"/>
+      <c r="W1" s="35"/>
+      <c r="X1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="Y1" s="28"/>
-      <c r="Z1" s="28"/>
-      <c r="AA1" s="28"/>
-      <c r="AB1" s="28"/>
-      <c r="AC1" s="28"/>
-      <c r="AD1" s="28"/>
-      <c r="AE1" s="28"/>
-      <c r="AF1" s="28"/>
-      <c r="AG1" s="28"/>
-      <c r="AH1" s="28"/>
-      <c r="AI1" s="28"/>
-      <c r="AJ1" s="28"/>
-      <c r="AK1" s="28"/>
-      <c r="AL1" s="29"/>
+      <c r="Y1" s="37"/>
+      <c r="Z1" s="37"/>
+      <c r="AA1" s="37"/>
+      <c r="AB1" s="37"/>
+      <c r="AC1" s="37"/>
+      <c r="AD1" s="37"/>
+      <c r="AE1" s="37"/>
+      <c r="AF1" s="37"/>
+      <c r="AG1" s="37"/>
+      <c r="AH1" s="37"/>
+      <c r="AI1" s="37"/>
+      <c r="AJ1" s="37"/>
+      <c r="AK1" s="37"/>
+      <c r="AL1" s="38"/>
     </row>
     <row r="2" spans="1:38" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="26"/>
-      <c r="T2" s="26"/>
-      <c r="U2" s="26"/>
-      <c r="V2" s="26"/>
-      <c r="W2" s="26"/>
-      <c r="X2" s="30"/>
-      <c r="Y2" s="31"/>
-      <c r="Z2" s="31"/>
-      <c r="AA2" s="31"/>
-      <c r="AB2" s="31"/>
-      <c r="AC2" s="31"/>
-      <c r="AD2" s="31"/>
-      <c r="AE2" s="31"/>
-      <c r="AF2" s="31"/>
-      <c r="AG2" s="31"/>
-      <c r="AH2" s="31"/>
-      <c r="AI2" s="31"/>
-      <c r="AJ2" s="31"/>
-      <c r="AK2" s="31"/>
-      <c r="AL2" s="32"/>
+      <c r="A2" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
+      <c r="T2" s="35"/>
+      <c r="U2" s="35"/>
+      <c r="V2" s="35"/>
+      <c r="W2" s="35"/>
+      <c r="X2" s="39"/>
+      <c r="Y2" s="40"/>
+      <c r="Z2" s="40"/>
+      <c r="AA2" s="40"/>
+      <c r="AB2" s="40"/>
+      <c r="AC2" s="40"/>
+      <c r="AD2" s="40"/>
+      <c r="AE2" s="40"/>
+      <c r="AF2" s="40"/>
+      <c r="AG2" s="40"/>
+      <c r="AH2" s="40"/>
+      <c r="AI2" s="40"/>
+      <c r="AJ2" s="40"/>
+      <c r="AK2" s="40"/>
+      <c r="AL2" s="41"/>
     </row>
     <row r="3" spans="1:38" s="1" customFormat="1" ht="42.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="40"/>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="40"/>
-      <c r="O3" s="40"/>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="40"/>
-      <c r="R3" s="40"/>
-      <c r="S3" s="40"/>
-      <c r="T3" s="40"/>
-      <c r="U3" s="40"/>
-      <c r="V3" s="40"/>
-      <c r="W3" s="40"/>
-      <c r="X3" s="40"/>
-      <c r="Y3" s="40"/>
-      <c r="Z3" s="40"/>
-      <c r="AA3" s="40"/>
-      <c r="AB3" s="40"/>
-      <c r="AC3" s="40"/>
-      <c r="AD3" s="40"/>
-      <c r="AE3" s="40"/>
-      <c r="AF3" s="40"/>
-      <c r="AG3" s="40"/>
-      <c r="AH3" s="41"/>
-      <c r="AI3" s="43" t="s">
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
+      <c r="L3" s="49"/>
+      <c r="M3" s="49"/>
+      <c r="N3" s="49"/>
+      <c r="O3" s="49"/>
+      <c r="P3" s="49"/>
+      <c r="Q3" s="49"/>
+      <c r="R3" s="49"/>
+      <c r="S3" s="49"/>
+      <c r="T3" s="49"/>
+      <c r="U3" s="49"/>
+      <c r="V3" s="49"/>
+      <c r="W3" s="49"/>
+      <c r="X3" s="49"/>
+      <c r="Y3" s="49"/>
+      <c r="Z3" s="49"/>
+      <c r="AA3" s="49"/>
+      <c r="AB3" s="49"/>
+      <c r="AC3" s="49"/>
+      <c r="AD3" s="49"/>
+      <c r="AE3" s="49"/>
+      <c r="AF3" s="49"/>
+      <c r="AG3" s="49"/>
+      <c r="AH3" s="50"/>
+      <c r="AI3" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="AJ3" s="54" t="s">
+      <c r="AJ3" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="AK3" s="42" t="s">
+      <c r="AK3" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="AL3" s="44" t="s">
+      <c r="AL3" s="53" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:38" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="34"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -2264,20 +2265,20 @@
       <c r="AF4" s="2"/>
       <c r="AG4" s="25"/>
       <c r="AH4" s="2"/>
-      <c r="AI4" s="43"/>
-      <c r="AJ4" s="55"/>
-      <c r="AK4" s="43"/>
-      <c r="AL4" s="45"/>
+      <c r="AI4" s="52"/>
+      <c r="AJ4" s="57"/>
+      <c r="AK4" s="52"/>
+      <c r="AL4" s="54"/>
     </row>
     <row r="5" spans="1:38" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="16" t="s">
         <v>21</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>22</v>
       </c>
       <c r="D5" s="24"/>
       <c r="E5" s="24"/>
@@ -3244,86 +3245,86 @@
       <c r="AL26" s="7"/>
     </row>
     <row r="27" spans="1:38" s="8" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="46" t="s">
+      <c r="A27" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B27" s="47"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="47"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="47"/>
-      <c r="I27" s="47"/>
-      <c r="J27" s="47"/>
-      <c r="K27" s="47"/>
-      <c r="L27" s="47"/>
-      <c r="M27" s="47"/>
-      <c r="N27" s="47"/>
-      <c r="O27" s="47"/>
-      <c r="P27" s="47"/>
-      <c r="Q27" s="47"/>
-      <c r="R27" s="47"/>
-      <c r="S27" s="47"/>
-      <c r="T27" s="47"/>
-      <c r="U27" s="47"/>
-      <c r="V27" s="47"/>
-      <c r="W27" s="47"/>
-      <c r="X27" s="47"/>
-      <c r="Y27" s="47"/>
-      <c r="Z27" s="47"/>
-      <c r="AA27" s="47"/>
-      <c r="AB27" s="47"/>
-      <c r="AC27" s="47"/>
-      <c r="AD27" s="47"/>
-      <c r="AE27" s="47"/>
-      <c r="AF27" s="47"/>
-      <c r="AG27" s="47"/>
-      <c r="AH27" s="47"/>
-      <c r="AI27" s="47"/>
-      <c r="AJ27" s="47"/>
-      <c r="AK27" s="47"/>
-      <c r="AL27" s="48"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="28"/>
+      <c r="J27" s="28"/>
+      <c r="K27" s="28"/>
+      <c r="L27" s="28"/>
+      <c r="M27" s="28"/>
+      <c r="N27" s="28"/>
+      <c r="O27" s="28"/>
+      <c r="P27" s="28"/>
+      <c r="Q27" s="28"/>
+      <c r="R27" s="28"/>
+      <c r="S27" s="28"/>
+      <c r="T27" s="28"/>
+      <c r="U27" s="28"/>
+      <c r="V27" s="28"/>
+      <c r="W27" s="28"/>
+      <c r="X27" s="28"/>
+      <c r="Y27" s="28"/>
+      <c r="Z27" s="28"/>
+      <c r="AA27" s="28"/>
+      <c r="AB27" s="28"/>
+      <c r="AC27" s="28"/>
+      <c r="AD27" s="28"/>
+      <c r="AE27" s="28"/>
+      <c r="AF27" s="28"/>
+      <c r="AG27" s="28"/>
+      <c r="AH27" s="28"/>
+      <c r="AI27" s="28"/>
+      <c r="AJ27" s="28"/>
+      <c r="AK27" s="28"/>
+      <c r="AL27" s="29"/>
     </row>
     <row r="28" spans="1:38" s="8" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A28" s="49"/>
-      <c r="B28" s="50"/>
-      <c r="C28" s="50"/>
-      <c r="D28" s="50"/>
-      <c r="E28" s="50"/>
-      <c r="F28" s="50"/>
-      <c r="G28" s="50"/>
-      <c r="H28" s="50"/>
-      <c r="I28" s="50"/>
-      <c r="J28" s="50"/>
-      <c r="K28" s="50"/>
-      <c r="L28" s="50"/>
-      <c r="M28" s="50"/>
-      <c r="N28" s="50"/>
-      <c r="O28" s="50"/>
-      <c r="P28" s="50"/>
-      <c r="Q28" s="50"/>
-      <c r="R28" s="50"/>
-      <c r="S28" s="50"/>
-      <c r="T28" s="50"/>
-      <c r="U28" s="50"/>
-      <c r="V28" s="50"/>
-      <c r="W28" s="50"/>
-      <c r="X28" s="50"/>
-      <c r="Y28" s="50"/>
-      <c r="Z28" s="50"/>
-      <c r="AA28" s="50"/>
-      <c r="AB28" s="50"/>
-      <c r="AC28" s="50"/>
-      <c r="AD28" s="50"/>
-      <c r="AE28" s="50"/>
-      <c r="AF28" s="50"/>
-      <c r="AG28" s="50"/>
-      <c r="AH28" s="50"/>
-      <c r="AI28" s="50"/>
-      <c r="AJ28" s="50"/>
-      <c r="AK28" s="50"/>
-      <c r="AL28" s="51"/>
+      <c r="A28" s="30"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="31"/>
+      <c r="J28" s="31"/>
+      <c r="K28" s="31"/>
+      <c r="L28" s="31"/>
+      <c r="M28" s="31"/>
+      <c r="N28" s="31"/>
+      <c r="O28" s="31"/>
+      <c r="P28" s="31"/>
+      <c r="Q28" s="31"/>
+      <c r="R28" s="31"/>
+      <c r="S28" s="31"/>
+      <c r="T28" s="31"/>
+      <c r="U28" s="31"/>
+      <c r="V28" s="31"/>
+      <c r="W28" s="31"/>
+      <c r="X28" s="31"/>
+      <c r="Y28" s="31"/>
+      <c r="Z28" s="31"/>
+      <c r="AA28" s="31"/>
+      <c r="AB28" s="31"/>
+      <c r="AC28" s="31"/>
+      <c r="AD28" s="31"/>
+      <c r="AE28" s="31"/>
+      <c r="AF28" s="31"/>
+      <c r="AG28" s="31"/>
+      <c r="AH28" s="31"/>
+      <c r="AI28" s="31"/>
+      <c r="AJ28" s="31"/>
+      <c r="AK28" s="31"/>
+      <c r="AL28" s="32"/>
     </row>
     <row r="29" spans="1:38" s="12" customFormat="1" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="9" t="s">
@@ -3331,67 +3332,61 @@
       </c>
       <c r="B29" s="9"/>
       <c r="C29" s="10" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
-      <c r="H29" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="I29" s="52"/>
-      <c r="J29" s="52"/>
+      <c r="H29" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="I29" s="33"/>
+      <c r="J29" s="33"/>
       <c r="K29" s="10"/>
       <c r="L29" s="10"/>
       <c r="M29" s="11"/>
       <c r="N29" s="11"/>
       <c r="O29" s="11"/>
-      <c r="P29" s="52" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q29" s="52"/>
-      <c r="R29" s="52"/>
+      <c r="P29" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q29" s="33"/>
+      <c r="R29" s="33"/>
       <c r="S29" s="11"/>
       <c r="T29" s="11"/>
       <c r="U29" s="11"/>
-      <c r="V29" s="52" t="s">
-        <v>17</v>
-      </c>
-      <c r="W29" s="52"/>
-      <c r="X29" s="52"/>
+      <c r="V29" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="W29" s="33"/>
+      <c r="X29" s="33"/>
       <c r="Y29" s="11"/>
       <c r="Z29" s="11"/>
       <c r="AA29" s="11"/>
-      <c r="AB29" s="52" t="s">
-        <v>18</v>
-      </c>
-      <c r="AC29" s="52"/>
-      <c r="AD29" s="52"/>
+      <c r="AB29" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="AC29" s="33"/>
+      <c r="AD29" s="33"/>
       <c r="AE29" s="11"/>
       <c r="AF29" s="11"/>
       <c r="AG29" s="11"/>
-      <c r="AH29" s="56" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI29" s="56"/>
+      <c r="AH29" s="55" t="s">
+        <v>18</v>
+      </c>
+      <c r="AI29" s="55"/>
       <c r="AJ29" s="10"/>
       <c r="AK29" s="10"/>
       <c r="AL29" s="10"/>
     </row>
     <row r="30" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A27:AL28"/>
-    <mergeCell ref="H29:J29"/>
-    <mergeCell ref="P29:R29"/>
-    <mergeCell ref="V29:X29"/>
-    <mergeCell ref="AB29:AD29"/>
-    <mergeCell ref="AH29:AI29"/>
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="X1:AL2"/>
     <mergeCell ref="A2:W2"/>
@@ -3403,6 +3398,12 @@
     <mergeCell ref="AJ3:AJ4"/>
     <mergeCell ref="AK3:AK4"/>
     <mergeCell ref="AL3:AL4"/>
+    <mergeCell ref="A27:AL28"/>
+    <mergeCell ref="H29:J29"/>
+    <mergeCell ref="P29:R29"/>
+    <mergeCell ref="V29:X29"/>
+    <mergeCell ref="AB29:AD29"/>
+    <mergeCell ref="AH29:AI29"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>

<commit_message>
Final: All report tags and print settings are now standardized and verified
</commit_message>
<xml_diff>
--- a/public/templates/drivebonus_template.xlsx
+++ b/public/templates/drivebonus_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\wordtoexcel\staff_manager\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DFB8E65-E0F0-4822-A652-3F98131D81B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7288ACB7-B75E-418A-A5D0-43F534C06BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="1" xr2:uid="{FE9DB102-5480-4C6F-9AE4-967FBD7E5687}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{FE9DB102-5480-4C6F-9AE4-967FBD7E5687}"/>
   </bookViews>
   <sheets>
     <sheet name="正駕" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="27">
   <si>
     <t>新北市政府環境保護局新店區清潔隊 隊員 駕駛安全獎金印領清冊</t>
   </si>
@@ -315,10 +315,6 @@
   </si>
   <si>
     <t>{{emp_id}}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>____{{year}}____年_{{month}}_月份</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -1324,7 +1320,7 @@
     </row>
     <row r="2" spans="1:38" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -1996,7 +1992,7 @@
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
@@ -2136,7 +2132,7 @@
     </row>
     <row r="2" spans="1:38" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -3336,7 +3332,7 @@
       </c>
       <c r="B29" s="9"/>
       <c r="C29" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>

</xml_diff>

<commit_message>
Final Update: Synchronized manually corrected Drive Bonus template and validated all export logic
</commit_message>
<xml_diff>
--- a/public/templates/drivebonus_template.xlsx
+++ b/public/templates/drivebonus_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\wordtoexcel\staff_manager\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7288ACB7-B75E-418A-A5D0-43F534C06BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A8B72E-3DBC-47F9-B1F9-B7D9204950A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{FE9DB102-5480-4C6F-9AE4-967FBD7E5687}"/>
   </bookViews>
@@ -541,19 +541,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top style="medium">
         <color indexed="64"/>
@@ -783,6 +770,19 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -790,22 +790,22 @@
   <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -815,45 +815,69 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -879,20 +903,20 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="distributed" vertical="center" indent="5"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="distributed" vertical="center" indent="5"/>
@@ -900,52 +924,28 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="distributed" vertical="center" indent="5"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="distributed" vertical="center" indent="5"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1275,151 +1275,151 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="44.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="27"/>
-      <c r="S1" s="27"/>
-      <c r="T1" s="27"/>
-      <c r="U1" s="27"/>
-      <c r="V1" s="27"/>
-      <c r="W1" s="27"/>
-      <c r="X1" s="28" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="35"/>
+      <c r="V1" s="35"/>
+      <c r="W1" s="35"/>
+      <c r="X1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="Y1" s="29"/>
-      <c r="Z1" s="29"/>
-      <c r="AA1" s="29"/>
-      <c r="AB1" s="29"/>
-      <c r="AC1" s="29"/>
-      <c r="AD1" s="29"/>
-      <c r="AE1" s="29"/>
-      <c r="AF1" s="29"/>
-      <c r="AG1" s="29"/>
-      <c r="AH1" s="29"/>
-      <c r="AI1" s="29"/>
-      <c r="AJ1" s="29"/>
-      <c r="AK1" s="29"/>
-      <c r="AL1" s="30"/>
+      <c r="Y1" s="37"/>
+      <c r="Z1" s="37"/>
+      <c r="AA1" s="37"/>
+      <c r="AB1" s="37"/>
+      <c r="AC1" s="37"/>
+      <c r="AD1" s="37"/>
+      <c r="AE1" s="37"/>
+      <c r="AF1" s="37"/>
+      <c r="AG1" s="37"/>
+      <c r="AH1" s="37"/>
+      <c r="AI1" s="37"/>
+      <c r="AJ1" s="37"/>
+      <c r="AK1" s="37"/>
+      <c r="AL1" s="38"/>
     </row>
     <row r="2" spans="1:38" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="27"/>
-      <c r="P2" s="27"/>
-      <c r="Q2" s="27"/>
-      <c r="R2" s="27"/>
-      <c r="S2" s="27"/>
-      <c r="T2" s="27"/>
-      <c r="U2" s="27"/>
-      <c r="V2" s="27"/>
-      <c r="W2" s="27"/>
-      <c r="X2" s="31"/>
-      <c r="Y2" s="32"/>
-      <c r="Z2" s="32"/>
-      <c r="AA2" s="32"/>
-      <c r="AB2" s="32"/>
-      <c r="AC2" s="32"/>
-      <c r="AD2" s="32"/>
-      <c r="AE2" s="32"/>
-      <c r="AF2" s="32"/>
-      <c r="AG2" s="32"/>
-      <c r="AH2" s="32"/>
-      <c r="AI2" s="32"/>
-      <c r="AJ2" s="32"/>
-      <c r="AK2" s="32"/>
-      <c r="AL2" s="33"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
+      <c r="T2" s="35"/>
+      <c r="U2" s="35"/>
+      <c r="V2" s="35"/>
+      <c r="W2" s="35"/>
+      <c r="X2" s="39"/>
+      <c r="Y2" s="40"/>
+      <c r="Z2" s="40"/>
+      <c r="AA2" s="40"/>
+      <c r="AB2" s="40"/>
+      <c r="AC2" s="40"/>
+      <c r="AD2" s="40"/>
+      <c r="AE2" s="40"/>
+      <c r="AF2" s="40"/>
+      <c r="AG2" s="40"/>
+      <c r="AH2" s="40"/>
+      <c r="AI2" s="40"/>
+      <c r="AJ2" s="40"/>
+      <c r="AK2" s="40"/>
+      <c r="AL2" s="41"/>
     </row>
     <row r="3" spans="1:38" s="1" customFormat="1" ht="42.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="38" t="s">
+      <c r="C3" s="57" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
-      <c r="L3" s="41"/>
-      <c r="M3" s="41"/>
-      <c r="N3" s="41"/>
-      <c r="O3" s="41"/>
-      <c r="P3" s="41"/>
-      <c r="Q3" s="41"/>
-      <c r="R3" s="41"/>
-      <c r="S3" s="41"/>
-      <c r="T3" s="41"/>
-      <c r="U3" s="41"/>
-      <c r="V3" s="41"/>
-      <c r="W3" s="41"/>
-      <c r="X3" s="41"/>
-      <c r="Y3" s="41"/>
-      <c r="Z3" s="41"/>
-      <c r="AA3" s="41"/>
-      <c r="AB3" s="41"/>
-      <c r="AC3" s="41"/>
-      <c r="AD3" s="41"/>
-      <c r="AE3" s="41"/>
-      <c r="AF3" s="41"/>
-      <c r="AG3" s="41"/>
-      <c r="AH3" s="42"/>
-      <c r="AI3" s="43" t="s">
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
+      <c r="L3" s="48"/>
+      <c r="M3" s="48"/>
+      <c r="N3" s="48"/>
+      <c r="O3" s="48"/>
+      <c r="P3" s="48"/>
+      <c r="Q3" s="48"/>
+      <c r="R3" s="48"/>
+      <c r="S3" s="48"/>
+      <c r="T3" s="48"/>
+      <c r="U3" s="48"/>
+      <c r="V3" s="48"/>
+      <c r="W3" s="48"/>
+      <c r="X3" s="48"/>
+      <c r="Y3" s="48"/>
+      <c r="Z3" s="48"/>
+      <c r="AA3" s="48"/>
+      <c r="AB3" s="48"/>
+      <c r="AC3" s="48"/>
+      <c r="AD3" s="48"/>
+      <c r="AE3" s="48"/>
+      <c r="AF3" s="48"/>
+      <c r="AG3" s="48"/>
+      <c r="AH3" s="49"/>
+      <c r="AI3" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="AJ3" s="43" t="s">
+      <c r="AJ3" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="AK3" s="43" t="s">
+      <c r="AK3" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="AL3" s="45" t="s">
+      <c r="AL3" s="52" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:38" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="35"/>
-      <c r="B4" s="37"/>
-      <c r="C4" s="39"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="46"/>
       <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
@@ -1453,10 +1453,10 @@
       <c r="AF4" s="2"/>
       <c r="AG4" s="2"/>
       <c r="AH4" s="2"/>
-      <c r="AI4" s="44"/>
-      <c r="AJ4" s="44"/>
-      <c r="AK4" s="44"/>
-      <c r="AL4" s="46"/>
+      <c r="AI4" s="51"/>
+      <c r="AJ4" s="51"/>
+      <c r="AK4" s="51"/>
+      <c r="AL4" s="53"/>
     </row>
     <row r="5" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="26" t="s">
@@ -1905,86 +1905,86 @@
       <c r="AL14" s="7"/>
     </row>
     <row r="15" spans="1:38" s="8" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="47" t="s">
+      <c r="A15" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="48"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="48"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="48"/>
-      <c r="G15" s="48"/>
-      <c r="H15" s="48"/>
-      <c r="I15" s="48"/>
-      <c r="J15" s="48"/>
-      <c r="K15" s="48"/>
-      <c r="L15" s="48"/>
-      <c r="M15" s="48"/>
-      <c r="N15" s="48"/>
-      <c r="O15" s="48"/>
-      <c r="P15" s="48"/>
-      <c r="Q15" s="48"/>
-      <c r="R15" s="48"/>
-      <c r="S15" s="48"/>
-      <c r="T15" s="48"/>
-      <c r="U15" s="48"/>
-      <c r="V15" s="48"/>
-      <c r="W15" s="48"/>
-      <c r="X15" s="48"/>
-      <c r="Y15" s="48"/>
-      <c r="Z15" s="48"/>
-      <c r="AA15" s="48"/>
-      <c r="AB15" s="48"/>
-      <c r="AC15" s="48"/>
-      <c r="AD15" s="48"/>
-      <c r="AE15" s="48"/>
-      <c r="AF15" s="48"/>
-      <c r="AG15" s="48"/>
-      <c r="AH15" s="48"/>
-      <c r="AI15" s="48"/>
-      <c r="AJ15" s="48"/>
-      <c r="AK15" s="48"/>
-      <c r="AL15" s="49"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="28"/>
+      <c r="K15" s="28"/>
+      <c r="L15" s="28"/>
+      <c r="M15" s="28"/>
+      <c r="N15" s="28"/>
+      <c r="O15" s="28"/>
+      <c r="P15" s="28"/>
+      <c r="Q15" s="28"/>
+      <c r="R15" s="28"/>
+      <c r="S15" s="28"/>
+      <c r="T15" s="28"/>
+      <c r="U15" s="28"/>
+      <c r="V15" s="28"/>
+      <c r="W15" s="28"/>
+      <c r="X15" s="28"/>
+      <c r="Y15" s="28"/>
+      <c r="Z15" s="28"/>
+      <c r="AA15" s="28"/>
+      <c r="AB15" s="28"/>
+      <c r="AC15" s="28"/>
+      <c r="AD15" s="28"/>
+      <c r="AE15" s="28"/>
+      <c r="AF15" s="28"/>
+      <c r="AG15" s="28"/>
+      <c r="AH15" s="28"/>
+      <c r="AI15" s="28"/>
+      <c r="AJ15" s="28"/>
+      <c r="AK15" s="28"/>
+      <c r="AL15" s="29"/>
     </row>
     <row r="16" spans="1:38" s="8" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A16" s="50"/>
-      <c r="B16" s="51"/>
-      <c r="C16" s="51"/>
-      <c r="D16" s="51"/>
-      <c r="E16" s="51"/>
-      <c r="F16" s="51"/>
-      <c r="G16" s="51"/>
-      <c r="H16" s="51"/>
-      <c r="I16" s="51"/>
-      <c r="J16" s="51"/>
-      <c r="K16" s="51"/>
-      <c r="L16" s="51"/>
-      <c r="M16" s="51"/>
-      <c r="N16" s="51"/>
-      <c r="O16" s="51"/>
-      <c r="P16" s="51"/>
-      <c r="Q16" s="51"/>
-      <c r="R16" s="51"/>
-      <c r="S16" s="51"/>
-      <c r="T16" s="51"/>
-      <c r="U16" s="51"/>
-      <c r="V16" s="51"/>
-      <c r="W16" s="51"/>
-      <c r="X16" s="51"/>
-      <c r="Y16" s="51"/>
-      <c r="Z16" s="51"/>
-      <c r="AA16" s="51"/>
-      <c r="AB16" s="51"/>
-      <c r="AC16" s="51"/>
-      <c r="AD16" s="51"/>
-      <c r="AE16" s="51"/>
-      <c r="AF16" s="51"/>
-      <c r="AG16" s="51"/>
-      <c r="AH16" s="51"/>
-      <c r="AI16" s="51"/>
-      <c r="AJ16" s="51"/>
-      <c r="AK16" s="51"/>
-      <c r="AL16" s="52"/>
+      <c r="A16" s="30"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="31"/>
+      <c r="L16" s="31"/>
+      <c r="M16" s="31"/>
+      <c r="N16" s="31"/>
+      <c r="O16" s="31"/>
+      <c r="P16" s="31"/>
+      <c r="Q16" s="31"/>
+      <c r="R16" s="31"/>
+      <c r="S16" s="31"/>
+      <c r="T16" s="31"/>
+      <c r="U16" s="31"/>
+      <c r="V16" s="31"/>
+      <c r="W16" s="31"/>
+      <c r="X16" s="31"/>
+      <c r="Y16" s="31"/>
+      <c r="Z16" s="31"/>
+      <c r="AA16" s="31"/>
+      <c r="AB16" s="31"/>
+      <c r="AC16" s="31"/>
+      <c r="AD16" s="31"/>
+      <c r="AE16" s="31"/>
+      <c r="AF16" s="31"/>
+      <c r="AG16" s="31"/>
+      <c r="AH16" s="31"/>
+      <c r="AI16" s="31"/>
+      <c r="AJ16" s="31"/>
+      <c r="AK16" s="31"/>
+      <c r="AL16" s="32"/>
     </row>
     <row r="17" spans="1:38" s="12" customFormat="1" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="9" t="s">
@@ -1998,56 +1998,50 @@
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
-      <c r="H17" s="53" t="s">
+      <c r="H17" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="I17" s="53"/>
-      <c r="J17" s="53"/>
+      <c r="I17" s="33"/>
+      <c r="J17" s="33"/>
       <c r="K17" s="10"/>
       <c r="L17" s="10"/>
       <c r="M17" s="11"/>
       <c r="N17" s="11"/>
       <c r="O17" s="11"/>
-      <c r="P17" s="53" t="s">
+      <c r="P17" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="Q17" s="53"/>
-      <c r="R17" s="53"/>
+      <c r="Q17" s="33"/>
+      <c r="R17" s="33"/>
       <c r="S17" s="11"/>
       <c r="T17" s="11"/>
       <c r="U17" s="11"/>
-      <c r="V17" s="53" t="s">
+      <c r="V17" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="W17" s="53"/>
-      <c r="X17" s="53"/>
+      <c r="W17" s="33"/>
+      <c r="X17" s="33"/>
       <c r="Y17" s="11"/>
       <c r="Z17" s="11"/>
       <c r="AA17" s="11"/>
-      <c r="AB17" s="53" t="s">
+      <c r="AB17" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="AC17" s="53"/>
-      <c r="AD17" s="53"/>
+      <c r="AC17" s="33"/>
+      <c r="AD17" s="33"/>
       <c r="AE17" s="11"/>
       <c r="AF17" s="11"/>
       <c r="AG17" s="11"/>
-      <c r="AH17" s="53" t="s">
+      <c r="AH17" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="AI17" s="54"/>
+      <c r="AI17" s="34"/>
       <c r="AJ17" s="10"/>
       <c r="AK17" s="10"/>
       <c r="AL17" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A15:AL16"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="P17:R17"/>
-    <mergeCell ref="V17:X17"/>
-    <mergeCell ref="AB17:AD17"/>
-    <mergeCell ref="AH17:AI17"/>
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="X1:AL2"/>
     <mergeCell ref="A2:W2"/>
@@ -2059,6 +2053,12 @@
     <mergeCell ref="AJ3:AJ4"/>
     <mergeCell ref="AK3:AK4"/>
     <mergeCell ref="AL3:AL4"/>
+    <mergeCell ref="A15:AL16"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="P17:R17"/>
+    <mergeCell ref="V17:X17"/>
+    <mergeCell ref="AB17:AD17"/>
+    <mergeCell ref="AH17:AI17"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2087,151 +2087,151 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="44.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="27"/>
-      <c r="S1" s="27"/>
-      <c r="T1" s="27"/>
-      <c r="U1" s="27"/>
-      <c r="V1" s="27"/>
-      <c r="W1" s="27"/>
-      <c r="X1" s="28" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="35"/>
+      <c r="V1" s="35"/>
+      <c r="W1" s="35"/>
+      <c r="X1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="Y1" s="29"/>
-      <c r="Z1" s="29"/>
-      <c r="AA1" s="29"/>
-      <c r="AB1" s="29"/>
-      <c r="AC1" s="29"/>
-      <c r="AD1" s="29"/>
-      <c r="AE1" s="29"/>
-      <c r="AF1" s="29"/>
-      <c r="AG1" s="29"/>
-      <c r="AH1" s="29"/>
-      <c r="AI1" s="29"/>
-      <c r="AJ1" s="29"/>
-      <c r="AK1" s="29"/>
-      <c r="AL1" s="30"/>
+      <c r="Y1" s="37"/>
+      <c r="Z1" s="37"/>
+      <c r="AA1" s="37"/>
+      <c r="AB1" s="37"/>
+      <c r="AC1" s="37"/>
+      <c r="AD1" s="37"/>
+      <c r="AE1" s="37"/>
+      <c r="AF1" s="37"/>
+      <c r="AG1" s="37"/>
+      <c r="AH1" s="37"/>
+      <c r="AI1" s="37"/>
+      <c r="AJ1" s="37"/>
+      <c r="AK1" s="37"/>
+      <c r="AL1" s="38"/>
     </row>
     <row r="2" spans="1:38" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="27"/>
-      <c r="P2" s="27"/>
-      <c r="Q2" s="27"/>
-      <c r="R2" s="27"/>
-      <c r="S2" s="27"/>
-      <c r="T2" s="27"/>
-      <c r="U2" s="27"/>
-      <c r="V2" s="27"/>
-      <c r="W2" s="27"/>
-      <c r="X2" s="31"/>
-      <c r="Y2" s="32"/>
-      <c r="Z2" s="32"/>
-      <c r="AA2" s="32"/>
-      <c r="AB2" s="32"/>
-      <c r="AC2" s="32"/>
-      <c r="AD2" s="32"/>
-      <c r="AE2" s="32"/>
-      <c r="AF2" s="32"/>
-      <c r="AG2" s="32"/>
-      <c r="AH2" s="32"/>
-      <c r="AI2" s="32"/>
-      <c r="AJ2" s="32"/>
-      <c r="AK2" s="32"/>
-      <c r="AL2" s="33"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
+      <c r="T2" s="35"/>
+      <c r="U2" s="35"/>
+      <c r="V2" s="35"/>
+      <c r="W2" s="35"/>
+      <c r="X2" s="39"/>
+      <c r="Y2" s="40"/>
+      <c r="Z2" s="40"/>
+      <c r="AA2" s="40"/>
+      <c r="AB2" s="40"/>
+      <c r="AC2" s="40"/>
+      <c r="AD2" s="40"/>
+      <c r="AE2" s="40"/>
+      <c r="AF2" s="40"/>
+      <c r="AG2" s="40"/>
+      <c r="AH2" s="40"/>
+      <c r="AI2" s="40"/>
+      <c r="AJ2" s="40"/>
+      <c r="AK2" s="40"/>
+      <c r="AL2" s="41"/>
     </row>
     <row r="3" spans="1:38" s="1" customFormat="1" ht="42.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="36" t="s">
+      <c r="C3" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
-      <c r="L3" s="41"/>
-      <c r="M3" s="41"/>
-      <c r="N3" s="41"/>
-      <c r="O3" s="41"/>
-      <c r="P3" s="41"/>
-      <c r="Q3" s="41"/>
-      <c r="R3" s="41"/>
-      <c r="S3" s="41"/>
-      <c r="T3" s="41"/>
-      <c r="U3" s="41"/>
-      <c r="V3" s="41"/>
-      <c r="W3" s="41"/>
-      <c r="X3" s="41"/>
-      <c r="Y3" s="41"/>
-      <c r="Z3" s="41"/>
-      <c r="AA3" s="41"/>
-      <c r="AB3" s="41"/>
-      <c r="AC3" s="41"/>
-      <c r="AD3" s="41"/>
-      <c r="AE3" s="41"/>
-      <c r="AF3" s="41"/>
-      <c r="AG3" s="41"/>
-      <c r="AH3" s="42"/>
-      <c r="AI3" s="44" t="s">
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
+      <c r="L3" s="48"/>
+      <c r="M3" s="48"/>
+      <c r="N3" s="48"/>
+      <c r="O3" s="48"/>
+      <c r="P3" s="48"/>
+      <c r="Q3" s="48"/>
+      <c r="R3" s="48"/>
+      <c r="S3" s="48"/>
+      <c r="T3" s="48"/>
+      <c r="U3" s="48"/>
+      <c r="V3" s="48"/>
+      <c r="W3" s="48"/>
+      <c r="X3" s="48"/>
+      <c r="Y3" s="48"/>
+      <c r="Z3" s="48"/>
+      <c r="AA3" s="48"/>
+      <c r="AB3" s="48"/>
+      <c r="AC3" s="48"/>
+      <c r="AD3" s="48"/>
+      <c r="AE3" s="48"/>
+      <c r="AF3" s="48"/>
+      <c r="AG3" s="48"/>
+      <c r="AH3" s="49"/>
+      <c r="AI3" s="51" t="s">
         <v>6</v>
       </c>
       <c r="AJ3" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="AK3" s="43" t="s">
+      <c r="AK3" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="AL3" s="45" t="s">
+      <c r="AL3" s="52" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:38" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="35"/>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
       <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
@@ -2265,10 +2265,10 @@
       <c r="AF4" s="2"/>
       <c r="AG4" s="25"/>
       <c r="AH4" s="2"/>
-      <c r="AI4" s="44"/>
+      <c r="AI4" s="51"/>
       <c r="AJ4" s="56"/>
-      <c r="AK4" s="44"/>
-      <c r="AL4" s="46"/>
+      <c r="AK4" s="51"/>
+      <c r="AL4" s="53"/>
     </row>
     <row r="5" spans="1:38" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
@@ -3245,86 +3245,86 @@
       <c r="AL26" s="7"/>
     </row>
     <row r="27" spans="1:38" s="8" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="47" t="s">
+      <c r="A27" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B27" s="48"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
-      <c r="I27" s="48"/>
-      <c r="J27" s="48"/>
-      <c r="K27" s="48"/>
-      <c r="L27" s="48"/>
-      <c r="M27" s="48"/>
-      <c r="N27" s="48"/>
-      <c r="O27" s="48"/>
-      <c r="P27" s="48"/>
-      <c r="Q27" s="48"/>
-      <c r="R27" s="48"/>
-      <c r="S27" s="48"/>
-      <c r="T27" s="48"/>
-      <c r="U27" s="48"/>
-      <c r="V27" s="48"/>
-      <c r="W27" s="48"/>
-      <c r="X27" s="48"/>
-      <c r="Y27" s="48"/>
-      <c r="Z27" s="48"/>
-      <c r="AA27" s="48"/>
-      <c r="AB27" s="48"/>
-      <c r="AC27" s="48"/>
-      <c r="AD27" s="48"/>
-      <c r="AE27" s="48"/>
-      <c r="AF27" s="48"/>
-      <c r="AG27" s="48"/>
-      <c r="AH27" s="48"/>
-      <c r="AI27" s="48"/>
-      <c r="AJ27" s="48"/>
-      <c r="AK27" s="48"/>
-      <c r="AL27" s="49"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="28"/>
+      <c r="J27" s="28"/>
+      <c r="K27" s="28"/>
+      <c r="L27" s="28"/>
+      <c r="M27" s="28"/>
+      <c r="N27" s="28"/>
+      <c r="O27" s="28"/>
+      <c r="P27" s="28"/>
+      <c r="Q27" s="28"/>
+      <c r="R27" s="28"/>
+      <c r="S27" s="28"/>
+      <c r="T27" s="28"/>
+      <c r="U27" s="28"/>
+      <c r="V27" s="28"/>
+      <c r="W27" s="28"/>
+      <c r="X27" s="28"/>
+      <c r="Y27" s="28"/>
+      <c r="Z27" s="28"/>
+      <c r="AA27" s="28"/>
+      <c r="AB27" s="28"/>
+      <c r="AC27" s="28"/>
+      <c r="AD27" s="28"/>
+      <c r="AE27" s="28"/>
+      <c r="AF27" s="28"/>
+      <c r="AG27" s="28"/>
+      <c r="AH27" s="28"/>
+      <c r="AI27" s="28"/>
+      <c r="AJ27" s="28"/>
+      <c r="AK27" s="28"/>
+      <c r="AL27" s="29"/>
     </row>
     <row r="28" spans="1:38" s="8" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A28" s="50"/>
-      <c r="B28" s="51"/>
-      <c r="C28" s="51"/>
-      <c r="D28" s="51"/>
-      <c r="E28" s="51"/>
-      <c r="F28" s="51"/>
-      <c r="G28" s="51"/>
-      <c r="H28" s="51"/>
-      <c r="I28" s="51"/>
-      <c r="J28" s="51"/>
-      <c r="K28" s="51"/>
-      <c r="L28" s="51"/>
-      <c r="M28" s="51"/>
-      <c r="N28" s="51"/>
-      <c r="O28" s="51"/>
-      <c r="P28" s="51"/>
-      <c r="Q28" s="51"/>
-      <c r="R28" s="51"/>
-      <c r="S28" s="51"/>
-      <c r="T28" s="51"/>
-      <c r="U28" s="51"/>
-      <c r="V28" s="51"/>
-      <c r="W28" s="51"/>
-      <c r="X28" s="51"/>
-      <c r="Y28" s="51"/>
-      <c r="Z28" s="51"/>
-      <c r="AA28" s="51"/>
-      <c r="AB28" s="51"/>
-      <c r="AC28" s="51"/>
-      <c r="AD28" s="51"/>
-      <c r="AE28" s="51"/>
-      <c r="AF28" s="51"/>
-      <c r="AG28" s="51"/>
-      <c r="AH28" s="51"/>
-      <c r="AI28" s="51"/>
-      <c r="AJ28" s="51"/>
-      <c r="AK28" s="51"/>
-      <c r="AL28" s="52"/>
+      <c r="A28" s="30"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="31"/>
+      <c r="J28" s="31"/>
+      <c r="K28" s="31"/>
+      <c r="L28" s="31"/>
+      <c r="M28" s="31"/>
+      <c r="N28" s="31"/>
+      <c r="O28" s="31"/>
+      <c r="P28" s="31"/>
+      <c r="Q28" s="31"/>
+      <c r="R28" s="31"/>
+      <c r="S28" s="31"/>
+      <c r="T28" s="31"/>
+      <c r="U28" s="31"/>
+      <c r="V28" s="31"/>
+      <c r="W28" s="31"/>
+      <c r="X28" s="31"/>
+      <c r="Y28" s="31"/>
+      <c r="Z28" s="31"/>
+      <c r="AA28" s="31"/>
+      <c r="AB28" s="31"/>
+      <c r="AC28" s="31"/>
+      <c r="AD28" s="31"/>
+      <c r="AE28" s="31"/>
+      <c r="AF28" s="31"/>
+      <c r="AG28" s="31"/>
+      <c r="AH28" s="31"/>
+      <c r="AI28" s="31"/>
+      <c r="AJ28" s="31"/>
+      <c r="AK28" s="31"/>
+      <c r="AL28" s="32"/>
     </row>
     <row r="29" spans="1:38" s="12" customFormat="1" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="9" t="s">
@@ -3338,44 +3338,44 @@
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
-      <c r="H29" s="53" t="s">
+      <c r="H29" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="I29" s="53"/>
-      <c r="J29" s="53"/>
+      <c r="I29" s="33"/>
+      <c r="J29" s="33"/>
       <c r="K29" s="10"/>
       <c r="L29" s="10"/>
       <c r="M29" s="11"/>
       <c r="N29" s="11"/>
       <c r="O29" s="11"/>
-      <c r="P29" s="53" t="s">
+      <c r="P29" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="Q29" s="53"/>
-      <c r="R29" s="53"/>
+      <c r="Q29" s="33"/>
+      <c r="R29" s="33"/>
       <c r="S29" s="11"/>
       <c r="T29" s="11"/>
       <c r="U29" s="11"/>
-      <c r="V29" s="53" t="s">
+      <c r="V29" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="W29" s="53"/>
-      <c r="X29" s="53"/>
+      <c r="W29" s="33"/>
+      <c r="X29" s="33"/>
       <c r="Y29" s="11"/>
       <c r="Z29" s="11"/>
       <c r="AA29" s="11"/>
-      <c r="AB29" s="53" t="s">
+      <c r="AB29" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="AC29" s="53"/>
-      <c r="AD29" s="53"/>
+      <c r="AC29" s="33"/>
+      <c r="AD29" s="33"/>
       <c r="AE29" s="11"/>
       <c r="AF29" s="11"/>
       <c r="AG29" s="11"/>
-      <c r="AH29" s="57" t="s">
+      <c r="AH29" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="AI29" s="57"/>
+      <c r="AI29" s="54"/>
       <c r="AJ29" s="10"/>
       <c r="AK29" s="10"/>
       <c r="AL29" s="10"/>
@@ -3387,12 +3387,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A27:AL28"/>
-    <mergeCell ref="H29:J29"/>
-    <mergeCell ref="P29:R29"/>
-    <mergeCell ref="V29:X29"/>
-    <mergeCell ref="AB29:AD29"/>
-    <mergeCell ref="AH29:AI29"/>
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="X1:AL2"/>
     <mergeCell ref="A2:W2"/>
@@ -3404,6 +3398,12 @@
     <mergeCell ref="AJ3:AJ4"/>
     <mergeCell ref="AK3:AK4"/>
     <mergeCell ref="AL3:AL4"/>
+    <mergeCell ref="A27:AL28"/>
+    <mergeCell ref="H29:J29"/>
+    <mergeCell ref="P29:R29"/>
+    <mergeCell ref="V29:X29"/>
+    <mergeCell ref="AB29:AD29"/>
+    <mergeCell ref="AH29:AI29"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>

<commit_message>
Fix: Upgraded border synchronization to robust nested loop to ensure no styled-only cells are skipped
</commit_message>
<xml_diff>
--- a/public/templates/drivebonus_template.xlsx
+++ b/public/templates/drivebonus_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\wordtoexcel\staff_manager\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A8B72E-3DBC-47F9-B1F9-B7D9204950A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E90D04-D626-4879-A95F-7C1B9974BBF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{FE9DB102-5480-4C6F-9AE4-967FBD7E5687}"/>
   </bookViews>
@@ -330,7 +330,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -422,6 +422,19 @@
       <family val="1"/>
       <charset val="136"/>
     </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -855,6 +868,60 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="distributed" vertical="center" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="distributed" vertical="center" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="distributed" vertical="center" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -879,73 +946,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="distributed" vertical="center" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="distributed" vertical="center" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="distributed" vertical="center" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1275,151 +1288,151 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="44.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-      <c r="X1" s="36" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="Y1" s="37"/>
-      <c r="Z1" s="37"/>
-      <c r="AA1" s="37"/>
-      <c r="AB1" s="37"/>
-      <c r="AC1" s="37"/>
-      <c r="AD1" s="37"/>
-      <c r="AE1" s="37"/>
-      <c r="AF1" s="37"/>
-      <c r="AG1" s="37"/>
-      <c r="AH1" s="37"/>
-      <c r="AI1" s="37"/>
-      <c r="AJ1" s="37"/>
-      <c r="AK1" s="37"/>
-      <c r="AL1" s="38"/>
+      <c r="Y1" s="29"/>
+      <c r="Z1" s="29"/>
+      <c r="AA1" s="29"/>
+      <c r="AB1" s="29"/>
+      <c r="AC1" s="29"/>
+      <c r="AD1" s="29"/>
+      <c r="AE1" s="29"/>
+      <c r="AF1" s="29"/>
+      <c r="AG1" s="29"/>
+      <c r="AH1" s="29"/>
+      <c r="AI1" s="29"/>
+      <c r="AJ1" s="29"/>
+      <c r="AK1" s="29"/>
+      <c r="AL1" s="30"/>
     </row>
     <row r="2" spans="1:38" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="35"/>
-      <c r="P2" s="35"/>
-      <c r="Q2" s="35"/>
-      <c r="R2" s="35"/>
-      <c r="S2" s="35"/>
-      <c r="T2" s="35"/>
-      <c r="U2" s="35"/>
-      <c r="V2" s="35"/>
-      <c r="W2" s="35"/>
-      <c r="X2" s="39"/>
-      <c r="Y2" s="40"/>
-      <c r="Z2" s="40"/>
-      <c r="AA2" s="40"/>
-      <c r="AB2" s="40"/>
-      <c r="AC2" s="40"/>
-      <c r="AD2" s="40"/>
-      <c r="AE2" s="40"/>
-      <c r="AF2" s="40"/>
-      <c r="AG2" s="40"/>
-      <c r="AH2" s="40"/>
-      <c r="AI2" s="40"/>
-      <c r="AJ2" s="40"/>
-      <c r="AK2" s="40"/>
-      <c r="AL2" s="41"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+      <c r="S2" s="27"/>
+      <c r="T2" s="27"/>
+      <c r="U2" s="27"/>
+      <c r="V2" s="27"/>
+      <c r="W2" s="27"/>
+      <c r="X2" s="31"/>
+      <c r="Y2" s="32"/>
+      <c r="Z2" s="32"/>
+      <c r="AA2" s="32"/>
+      <c r="AB2" s="32"/>
+      <c r="AC2" s="32"/>
+      <c r="AD2" s="32"/>
+      <c r="AE2" s="32"/>
+      <c r="AF2" s="32"/>
+      <c r="AG2" s="32"/>
+      <c r="AH2" s="32"/>
+      <c r="AI2" s="32"/>
+      <c r="AJ2" s="32"/>
+      <c r="AK2" s="32"/>
+      <c r="AL2" s="33"/>
     </row>
     <row r="3" spans="1:38" s="1" customFormat="1" ht="42.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="57" t="s">
+      <c r="C3" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="47" t="s">
+      <c r="D3" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-      <c r="L3" s="48"/>
-      <c r="M3" s="48"/>
-      <c r="N3" s="48"/>
-      <c r="O3" s="48"/>
-      <c r="P3" s="48"/>
-      <c r="Q3" s="48"/>
-      <c r="R3" s="48"/>
-      <c r="S3" s="48"/>
-      <c r="T3" s="48"/>
-      <c r="U3" s="48"/>
-      <c r="V3" s="48"/>
-      <c r="W3" s="48"/>
-      <c r="X3" s="48"/>
-      <c r="Y3" s="48"/>
-      <c r="Z3" s="48"/>
-      <c r="AA3" s="48"/>
-      <c r="AB3" s="48"/>
-      <c r="AC3" s="48"/>
-      <c r="AD3" s="48"/>
-      <c r="AE3" s="48"/>
-      <c r="AF3" s="48"/>
-      <c r="AG3" s="48"/>
-      <c r="AH3" s="49"/>
-      <c r="AI3" s="50" t="s">
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="39"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="39"/>
+      <c r="T3" s="39"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="39"/>
+      <c r="W3" s="39"/>
+      <c r="X3" s="39"/>
+      <c r="Y3" s="39"/>
+      <c r="Z3" s="39"/>
+      <c r="AA3" s="39"/>
+      <c r="AB3" s="39"/>
+      <c r="AC3" s="39"/>
+      <c r="AD3" s="39"/>
+      <c r="AE3" s="39"/>
+      <c r="AF3" s="39"/>
+      <c r="AG3" s="39"/>
+      <c r="AH3" s="40"/>
+      <c r="AI3" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="AJ3" s="50" t="s">
+      <c r="AJ3" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="AK3" s="50" t="s">
+      <c r="AK3" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="AL3" s="52" t="s">
+      <c r="AL3" s="43" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:38" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="43"/>
-      <c r="B4" s="45"/>
-      <c r="C4" s="46"/>
+      <c r="A4" s="35"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="57"/>
       <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
@@ -1453,10 +1466,10 @@
       <c r="AF4" s="2"/>
       <c r="AG4" s="2"/>
       <c r="AH4" s="2"/>
-      <c r="AI4" s="51"/>
-      <c r="AJ4" s="51"/>
-      <c r="AK4" s="51"/>
-      <c r="AL4" s="53"/>
+      <c r="AI4" s="42"/>
+      <c r="AJ4" s="42"/>
+      <c r="AK4" s="42"/>
+      <c r="AL4" s="44"/>
     </row>
     <row r="5" spans="1:38" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="26" t="s">
@@ -1905,86 +1918,86 @@
       <c r="AL14" s="7"/>
     </row>
     <row r="15" spans="1:38" s="8" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="28"/>
-      <c r="J15" s="28"/>
-      <c r="K15" s="28"/>
-      <c r="L15" s="28"/>
-      <c r="M15" s="28"/>
-      <c r="N15" s="28"/>
-      <c r="O15" s="28"/>
-      <c r="P15" s="28"/>
-      <c r="Q15" s="28"/>
-      <c r="R15" s="28"/>
-      <c r="S15" s="28"/>
-      <c r="T15" s="28"/>
-      <c r="U15" s="28"/>
-      <c r="V15" s="28"/>
-      <c r="W15" s="28"/>
-      <c r="X15" s="28"/>
-      <c r="Y15" s="28"/>
-      <c r="Z15" s="28"/>
-      <c r="AA15" s="28"/>
-      <c r="AB15" s="28"/>
-      <c r="AC15" s="28"/>
-      <c r="AD15" s="28"/>
-      <c r="AE15" s="28"/>
-      <c r="AF15" s="28"/>
-      <c r="AG15" s="28"/>
-      <c r="AH15" s="28"/>
-      <c r="AI15" s="28"/>
-      <c r="AJ15" s="28"/>
-      <c r="AK15" s="28"/>
-      <c r="AL15" s="29"/>
+      <c r="B15" s="46"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="46"/>
+      <c r="E15" s="46"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="46"/>
+      <c r="K15" s="46"/>
+      <c r="L15" s="46"/>
+      <c r="M15" s="46"/>
+      <c r="N15" s="46"/>
+      <c r="O15" s="46"/>
+      <c r="P15" s="46"/>
+      <c r="Q15" s="46"/>
+      <c r="R15" s="46"/>
+      <c r="S15" s="46"/>
+      <c r="T15" s="46"/>
+      <c r="U15" s="46"/>
+      <c r="V15" s="46"/>
+      <c r="W15" s="46"/>
+      <c r="X15" s="46"/>
+      <c r="Y15" s="46"/>
+      <c r="Z15" s="46"/>
+      <c r="AA15" s="46"/>
+      <c r="AB15" s="46"/>
+      <c r="AC15" s="46"/>
+      <c r="AD15" s="46"/>
+      <c r="AE15" s="46"/>
+      <c r="AF15" s="46"/>
+      <c r="AG15" s="46"/>
+      <c r="AH15" s="46"/>
+      <c r="AI15" s="46"/>
+      <c r="AJ15" s="46"/>
+      <c r="AK15" s="46"/>
+      <c r="AL15" s="47"/>
     </row>
     <row r="16" spans="1:38" s="8" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A16" s="30"/>
-      <c r="B16" s="31"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="31"/>
-      <c r="I16" s="31"/>
-      <c r="J16" s="31"/>
-      <c r="K16" s="31"/>
-      <c r="L16" s="31"/>
-      <c r="M16" s="31"/>
-      <c r="N16" s="31"/>
-      <c r="O16" s="31"/>
-      <c r="P16" s="31"/>
-      <c r="Q16" s="31"/>
-      <c r="R16" s="31"/>
-      <c r="S16" s="31"/>
-      <c r="T16" s="31"/>
-      <c r="U16" s="31"/>
-      <c r="V16" s="31"/>
-      <c r="W16" s="31"/>
-      <c r="X16" s="31"/>
-      <c r="Y16" s="31"/>
-      <c r="Z16" s="31"/>
-      <c r="AA16" s="31"/>
-      <c r="AB16" s="31"/>
-      <c r="AC16" s="31"/>
-      <c r="AD16" s="31"/>
-      <c r="AE16" s="31"/>
-      <c r="AF16" s="31"/>
-      <c r="AG16" s="31"/>
-      <c r="AH16" s="31"/>
-      <c r="AI16" s="31"/>
-      <c r="AJ16" s="31"/>
-      <c r="AK16" s="31"/>
-      <c r="AL16" s="32"/>
+      <c r="A16" s="48"/>
+      <c r="B16" s="49"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="49"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="49"/>
+      <c r="I16" s="49"/>
+      <c r="J16" s="49"/>
+      <c r="K16" s="49"/>
+      <c r="L16" s="49"/>
+      <c r="M16" s="49"/>
+      <c r="N16" s="49"/>
+      <c r="O16" s="49"/>
+      <c r="P16" s="49"/>
+      <c r="Q16" s="49"/>
+      <c r="R16" s="49"/>
+      <c r="S16" s="49"/>
+      <c r="T16" s="49"/>
+      <c r="U16" s="49"/>
+      <c r="V16" s="49"/>
+      <c r="W16" s="49"/>
+      <c r="X16" s="49"/>
+      <c r="Y16" s="49"/>
+      <c r="Z16" s="49"/>
+      <c r="AA16" s="49"/>
+      <c r="AB16" s="49"/>
+      <c r="AC16" s="49"/>
+      <c r="AD16" s="49"/>
+      <c r="AE16" s="49"/>
+      <c r="AF16" s="49"/>
+      <c r="AG16" s="49"/>
+      <c r="AH16" s="49"/>
+      <c r="AI16" s="49"/>
+      <c r="AJ16" s="49"/>
+      <c r="AK16" s="49"/>
+      <c r="AL16" s="50"/>
     </row>
     <row r="17" spans="1:38" s="12" customFormat="1" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="9" t="s">
@@ -1998,50 +2011,56 @@
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
-      <c r="H17" s="33" t="s">
+      <c r="H17" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="I17" s="33"/>
-      <c r="J17" s="33"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="51"/>
       <c r="K17" s="10"/>
       <c r="L17" s="10"/>
       <c r="M17" s="11"/>
       <c r="N17" s="11"/>
       <c r="O17" s="11"/>
-      <c r="P17" s="33" t="s">
+      <c r="P17" s="51" t="s">
         <v>15</v>
       </c>
-      <c r="Q17" s="33"/>
-      <c r="R17" s="33"/>
+      <c r="Q17" s="51"/>
+      <c r="R17" s="51"/>
       <c r="S17" s="11"/>
       <c r="T17" s="11"/>
       <c r="U17" s="11"/>
-      <c r="V17" s="33" t="s">
+      <c r="V17" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="W17" s="33"/>
-      <c r="X17" s="33"/>
+      <c r="W17" s="51"/>
+      <c r="X17" s="51"/>
       <c r="Y17" s="11"/>
       <c r="Z17" s="11"/>
       <c r="AA17" s="11"/>
-      <c r="AB17" s="33" t="s">
+      <c r="AB17" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="AC17" s="33"/>
-      <c r="AD17" s="33"/>
+      <c r="AC17" s="51"/>
+      <c r="AD17" s="51"/>
       <c r="AE17" s="11"/>
       <c r="AF17" s="11"/>
       <c r="AG17" s="11"/>
-      <c r="AH17" s="33" t="s">
+      <c r="AH17" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="AI17" s="34"/>
+      <c r="AI17" s="52"/>
       <c r="AJ17" s="10"/>
       <c r="AK17" s="10"/>
       <c r="AL17" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A15:AL16"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="P17:R17"/>
+    <mergeCell ref="V17:X17"/>
+    <mergeCell ref="AB17:AD17"/>
+    <mergeCell ref="AH17:AI17"/>
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="X1:AL2"/>
     <mergeCell ref="A2:W2"/>
@@ -2053,12 +2072,6 @@
     <mergeCell ref="AJ3:AJ4"/>
     <mergeCell ref="AK3:AK4"/>
     <mergeCell ref="AL3:AL4"/>
-    <mergeCell ref="A15:AL16"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="P17:R17"/>
-    <mergeCell ref="V17:X17"/>
-    <mergeCell ref="AB17:AD17"/>
-    <mergeCell ref="AH17:AI17"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2087,151 +2100,151 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="44.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-      <c r="X1" s="36" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="Y1" s="37"/>
-      <c r="Z1" s="37"/>
-      <c r="AA1" s="37"/>
-      <c r="AB1" s="37"/>
-      <c r="AC1" s="37"/>
-      <c r="AD1" s="37"/>
-      <c r="AE1" s="37"/>
-      <c r="AF1" s="37"/>
-      <c r="AG1" s="37"/>
-      <c r="AH1" s="37"/>
-      <c r="AI1" s="37"/>
-      <c r="AJ1" s="37"/>
-      <c r="AK1" s="37"/>
-      <c r="AL1" s="38"/>
+      <c r="Y1" s="29"/>
+      <c r="Z1" s="29"/>
+      <c r="AA1" s="29"/>
+      <c r="AB1" s="29"/>
+      <c r="AC1" s="29"/>
+      <c r="AD1" s="29"/>
+      <c r="AE1" s="29"/>
+      <c r="AF1" s="29"/>
+      <c r="AG1" s="29"/>
+      <c r="AH1" s="29"/>
+      <c r="AI1" s="29"/>
+      <c r="AJ1" s="29"/>
+      <c r="AK1" s="29"/>
+      <c r="AL1" s="30"/>
     </row>
     <row r="2" spans="1:38" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="35"/>
-      <c r="P2" s="35"/>
-      <c r="Q2" s="35"/>
-      <c r="R2" s="35"/>
-      <c r="S2" s="35"/>
-      <c r="T2" s="35"/>
-      <c r="U2" s="35"/>
-      <c r="V2" s="35"/>
-      <c r="W2" s="35"/>
-      <c r="X2" s="39"/>
-      <c r="Y2" s="40"/>
-      <c r="Z2" s="40"/>
-      <c r="AA2" s="40"/>
-      <c r="AB2" s="40"/>
-      <c r="AC2" s="40"/>
-      <c r="AD2" s="40"/>
-      <c r="AE2" s="40"/>
-      <c r="AF2" s="40"/>
-      <c r="AG2" s="40"/>
-      <c r="AH2" s="40"/>
-      <c r="AI2" s="40"/>
-      <c r="AJ2" s="40"/>
-      <c r="AK2" s="40"/>
-      <c r="AL2" s="41"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+      <c r="S2" s="27"/>
+      <c r="T2" s="27"/>
+      <c r="U2" s="27"/>
+      <c r="V2" s="27"/>
+      <c r="W2" s="27"/>
+      <c r="X2" s="31"/>
+      <c r="Y2" s="32"/>
+      <c r="Z2" s="32"/>
+      <c r="AA2" s="32"/>
+      <c r="AB2" s="32"/>
+      <c r="AC2" s="32"/>
+      <c r="AD2" s="32"/>
+      <c r="AE2" s="32"/>
+      <c r="AF2" s="32"/>
+      <c r="AG2" s="32"/>
+      <c r="AH2" s="32"/>
+      <c r="AI2" s="32"/>
+      <c r="AJ2" s="32"/>
+      <c r="AK2" s="32"/>
+      <c r="AL2" s="33"/>
     </row>
     <row r="3" spans="1:38" s="1" customFormat="1" ht="42.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="47" t="s">
+      <c r="D3" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-      <c r="L3" s="48"/>
-      <c r="M3" s="48"/>
-      <c r="N3" s="48"/>
-      <c r="O3" s="48"/>
-      <c r="P3" s="48"/>
-      <c r="Q3" s="48"/>
-      <c r="R3" s="48"/>
-      <c r="S3" s="48"/>
-      <c r="T3" s="48"/>
-      <c r="U3" s="48"/>
-      <c r="V3" s="48"/>
-      <c r="W3" s="48"/>
-      <c r="X3" s="48"/>
-      <c r="Y3" s="48"/>
-      <c r="Z3" s="48"/>
-      <c r="AA3" s="48"/>
-      <c r="AB3" s="48"/>
-      <c r="AC3" s="48"/>
-      <c r="AD3" s="48"/>
-      <c r="AE3" s="48"/>
-      <c r="AF3" s="48"/>
-      <c r="AG3" s="48"/>
-      <c r="AH3" s="49"/>
-      <c r="AI3" s="51" t="s">
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="39"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="39"/>
+      <c r="T3" s="39"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="39"/>
+      <c r="W3" s="39"/>
+      <c r="X3" s="39"/>
+      <c r="Y3" s="39"/>
+      <c r="Z3" s="39"/>
+      <c r="AA3" s="39"/>
+      <c r="AB3" s="39"/>
+      <c r="AC3" s="39"/>
+      <c r="AD3" s="39"/>
+      <c r="AE3" s="39"/>
+      <c r="AF3" s="39"/>
+      <c r="AG3" s="39"/>
+      <c r="AH3" s="40"/>
+      <c r="AI3" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="AJ3" s="55" t="s">
+      <c r="AJ3" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="AK3" s="50" t="s">
+      <c r="AK3" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="AL3" s="52" t="s">
+      <c r="AL3" s="43" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:38" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="43"/>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
+      <c r="A4" s="35"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="37"/>
       <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
@@ -2265,10 +2278,10 @@
       <c r="AF4" s="2"/>
       <c r="AG4" s="25"/>
       <c r="AH4" s="2"/>
-      <c r="AI4" s="51"/>
-      <c r="AJ4" s="56"/>
-      <c r="AK4" s="51"/>
-      <c r="AL4" s="53"/>
+      <c r="AI4" s="42"/>
+      <c r="AJ4" s="54"/>
+      <c r="AK4" s="42"/>
+      <c r="AL4" s="44"/>
     </row>
     <row r="5" spans="1:38" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
@@ -3245,86 +3258,86 @@
       <c r="AL26" s="7"/>
     </row>
     <row r="27" spans="1:38" s="8" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="27" t="s">
+      <c r="A27" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="28"/>
-      <c r="H27" s="28"/>
-      <c r="I27" s="28"/>
-      <c r="J27" s="28"/>
-      <c r="K27" s="28"/>
-      <c r="L27" s="28"/>
-      <c r="M27" s="28"/>
-      <c r="N27" s="28"/>
-      <c r="O27" s="28"/>
-      <c r="P27" s="28"/>
-      <c r="Q27" s="28"/>
-      <c r="R27" s="28"/>
-      <c r="S27" s="28"/>
-      <c r="T27" s="28"/>
-      <c r="U27" s="28"/>
-      <c r="V27" s="28"/>
-      <c r="W27" s="28"/>
-      <c r="X27" s="28"/>
-      <c r="Y27" s="28"/>
-      <c r="Z27" s="28"/>
-      <c r="AA27" s="28"/>
-      <c r="AB27" s="28"/>
-      <c r="AC27" s="28"/>
-      <c r="AD27" s="28"/>
-      <c r="AE27" s="28"/>
-      <c r="AF27" s="28"/>
-      <c r="AG27" s="28"/>
-      <c r="AH27" s="28"/>
-      <c r="AI27" s="28"/>
-      <c r="AJ27" s="28"/>
-      <c r="AK27" s="28"/>
-      <c r="AL27" s="29"/>
+      <c r="B27" s="46"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="46"/>
+      <c r="I27" s="46"/>
+      <c r="J27" s="46"/>
+      <c r="K27" s="46"/>
+      <c r="L27" s="46"/>
+      <c r="M27" s="46"/>
+      <c r="N27" s="46"/>
+      <c r="O27" s="46"/>
+      <c r="P27" s="46"/>
+      <c r="Q27" s="46"/>
+      <c r="R27" s="46"/>
+      <c r="S27" s="46"/>
+      <c r="T27" s="46"/>
+      <c r="U27" s="46"/>
+      <c r="V27" s="46"/>
+      <c r="W27" s="46"/>
+      <c r="X27" s="46"/>
+      <c r="Y27" s="46"/>
+      <c r="Z27" s="46"/>
+      <c r="AA27" s="46"/>
+      <c r="AB27" s="46"/>
+      <c r="AC27" s="46"/>
+      <c r="AD27" s="46"/>
+      <c r="AE27" s="46"/>
+      <c r="AF27" s="46"/>
+      <c r="AG27" s="46"/>
+      <c r="AH27" s="46"/>
+      <c r="AI27" s="46"/>
+      <c r="AJ27" s="46"/>
+      <c r="AK27" s="46"/>
+      <c r="AL27" s="47"/>
     </row>
     <row r="28" spans="1:38" s="8" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A28" s="30"/>
-      <c r="B28" s="31"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="31"/>
-      <c r="I28" s="31"/>
-      <c r="J28" s="31"/>
-      <c r="K28" s="31"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="31"/>
-      <c r="O28" s="31"/>
-      <c r="P28" s="31"/>
-      <c r="Q28" s="31"/>
-      <c r="R28" s="31"/>
-      <c r="S28" s="31"/>
-      <c r="T28" s="31"/>
-      <c r="U28" s="31"/>
-      <c r="V28" s="31"/>
-      <c r="W28" s="31"/>
-      <c r="X28" s="31"/>
-      <c r="Y28" s="31"/>
-      <c r="Z28" s="31"/>
-      <c r="AA28" s="31"/>
-      <c r="AB28" s="31"/>
-      <c r="AC28" s="31"/>
-      <c r="AD28" s="31"/>
-      <c r="AE28" s="31"/>
-      <c r="AF28" s="31"/>
-      <c r="AG28" s="31"/>
-      <c r="AH28" s="31"/>
-      <c r="AI28" s="31"/>
-      <c r="AJ28" s="31"/>
-      <c r="AK28" s="31"/>
-      <c r="AL28" s="32"/>
+      <c r="A28" s="48"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="49"/>
+      <c r="F28" s="49"/>
+      <c r="G28" s="49"/>
+      <c r="H28" s="49"/>
+      <c r="I28" s="49"/>
+      <c r="J28" s="49"/>
+      <c r="K28" s="49"/>
+      <c r="L28" s="49"/>
+      <c r="M28" s="49"/>
+      <c r="N28" s="49"/>
+      <c r="O28" s="49"/>
+      <c r="P28" s="49"/>
+      <c r="Q28" s="49"/>
+      <c r="R28" s="49"/>
+      <c r="S28" s="49"/>
+      <c r="T28" s="49"/>
+      <c r="U28" s="49"/>
+      <c r="V28" s="49"/>
+      <c r="W28" s="49"/>
+      <c r="X28" s="49"/>
+      <c r="Y28" s="49"/>
+      <c r="Z28" s="49"/>
+      <c r="AA28" s="49"/>
+      <c r="AB28" s="49"/>
+      <c r="AC28" s="49"/>
+      <c r="AD28" s="49"/>
+      <c r="AE28" s="49"/>
+      <c r="AF28" s="49"/>
+      <c r="AG28" s="49"/>
+      <c r="AH28" s="49"/>
+      <c r="AI28" s="49"/>
+      <c r="AJ28" s="49"/>
+      <c r="AK28" s="49"/>
+      <c r="AL28" s="50"/>
     </row>
     <row r="29" spans="1:38" s="12" customFormat="1" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="9" t="s">
@@ -3338,44 +3351,44 @@
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
-      <c r="H29" s="33" t="s">
+      <c r="H29" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="I29" s="33"/>
-      <c r="J29" s="33"/>
+      <c r="I29" s="51"/>
+      <c r="J29" s="51"/>
       <c r="K29" s="10"/>
       <c r="L29" s="10"/>
       <c r="M29" s="11"/>
       <c r="N29" s="11"/>
       <c r="O29" s="11"/>
-      <c r="P29" s="33" t="s">
+      <c r="P29" s="51" t="s">
         <v>15</v>
       </c>
-      <c r="Q29" s="33"/>
-      <c r="R29" s="33"/>
+      <c r="Q29" s="51"/>
+      <c r="R29" s="51"/>
       <c r="S29" s="11"/>
       <c r="T29" s="11"/>
       <c r="U29" s="11"/>
-      <c r="V29" s="33" t="s">
+      <c r="V29" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="W29" s="33"/>
-      <c r="X29" s="33"/>
+      <c r="W29" s="51"/>
+      <c r="X29" s="51"/>
       <c r="Y29" s="11"/>
       <c r="Z29" s="11"/>
       <c r="AA29" s="11"/>
-      <c r="AB29" s="33" t="s">
+      <c r="AB29" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="AC29" s="33"/>
-      <c r="AD29" s="33"/>
+      <c r="AC29" s="51"/>
+      <c r="AD29" s="51"/>
       <c r="AE29" s="11"/>
       <c r="AF29" s="11"/>
       <c r="AG29" s="11"/>
-      <c r="AH29" s="54" t="s">
+      <c r="AH29" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="AI29" s="54"/>
+      <c r="AI29" s="55"/>
       <c r="AJ29" s="10"/>
       <c r="AK29" s="10"/>
       <c r="AL29" s="10"/>
@@ -3387,6 +3400,12 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A27:AL28"/>
+    <mergeCell ref="H29:J29"/>
+    <mergeCell ref="P29:R29"/>
+    <mergeCell ref="V29:X29"/>
+    <mergeCell ref="AB29:AD29"/>
+    <mergeCell ref="AH29:AI29"/>
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="X1:AL2"/>
     <mergeCell ref="A2:W2"/>
@@ -3398,12 +3417,6 @@
     <mergeCell ref="AJ3:AJ4"/>
     <mergeCell ref="AK3:AK4"/>
     <mergeCell ref="AL3:AL4"/>
-    <mergeCell ref="A27:AL28"/>
-    <mergeCell ref="H29:J29"/>
-    <mergeCell ref="P29:R29"/>
-    <mergeCell ref="V29:X29"/>
-    <mergeCell ref="AB29:AD29"/>
-    <mergeCell ref="AH29:AI29"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>